<commit_message>
Alinea el acta de constitución (v3) con la línea base de costos
El acta v3 describe la implementación del CRM (software, 4 meses, hitos
H0-H5) y autoriza S/ 42 200. La línea base de costos se recalcula con
tarifas de perfil junior: presupuesto S/ 42 066, dentro de lo autorizado.
Se actualizan la sección de costos, el Excel y la página del acta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LWjTm2rp677phoNoYSvNSp
</commit_message>
<xml_diff>
--- a/docs/Costos_CRM_Essenza.xlsx
+++ b/docs/Costos_CRM_Essenza.xlsx
@@ -67,12 +67,24 @@
         </r>
       </text>
     </comment>
+    <comment ref="B20" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Monto de orden de magnitud aprobado en el acta ESSENZA-CRM-2026-001 (sección 10).</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="307">
   <si>
     <t xml:space="preserve">Línea base de costos — CRM Predictivo y Retención Postventa · Essenza SPA</t>
   </si>
@@ -137,6 +149,18 @@
     <t xml:space="preserve">Línea base + reserva de gestión</t>
   </si>
   <si>
+    <t xml:space="preserve">Presupuesto autorizado en el acta (v3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orden de magnitud aprobado en el acta de constitución</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holgura frente al acta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autorizado − presupuesto del proyecto</t>
+  </si>
+  <si>
     <t xml:space="preserve">Leyenda</t>
   </si>
   <si>
@@ -296,7 +320,7 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuente de los sueldos: valores de referencia del mercado de Lima para perfiles TI junior/semisenior (supuesto del equipo, no cotización). Los roles internos (administradora y dueña) se valorizan con su costo de oportunidad.</t>
+    <t xml:space="preserve">Fuente de los sueldos: valores de referencia del mercado de Lima para perfiles TI junior (supuesto del equipo, no cotización). Los roles internos (administradora y dueña) se valorizan con su costo de oportunidad.</t>
   </si>
   <si>
     <t xml:space="preserve">Materiales, equipos y gastos que no son horas del equipo. Montos en azul = entrada.</t>
@@ -731,6 +755,15 @@
     <t xml:space="preserve">+ Reserva de gestión (S/)</t>
   </si>
   <si>
+    <t xml:space="preserve">Presupuesto autorizado en el acta de constitución (v3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holgura frente al acta (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tope con tolerancia del acta (+10 %)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Curva S — valor planificado (PV) acumulado por semana</t>
   </si>
   <si>
@@ -806,7 +839,7 @@
     <t xml:space="preserve">Sobrecosto observado (AC / EV)</t>
   </si>
   <si>
-    <t xml:space="preserve">Supuesto del ejemplo: se gastó 5 % más de lo ganado</t>
+    <t xml:space="preserve">Supuesto del ejemplo: se gastó 6 % más de lo ganado</t>
   </si>
   <si>
     <t xml:space="preserve">AC — costo real</t>
@@ -1359,6 +1392,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1384,10 +1421,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1602,28 +1635,28 @@
                 <c:formatCode>"S/ "#,##0;[RED]"-S/ "#,##0;\-</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>14680</c:v>
+                  <c:v>9048</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5104</c:v>
+                  <c:v>3304</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8481</c:v>
+                  <c:v>4905</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5721</c:v>
+                  <c:v>3575</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4752</c:v>
+                  <c:v>2880</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5214</c:v>
+                  <c:v>3184</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3840</c:v>
+                  <c:v>2544</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>11962</c:v>
+                  <c:v>8098</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1631,11 +1664,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="57187827"/>
-        <c:axId val="95604837"/>
+        <c:axId val="52922887"/>
+        <c:axId val="62129246"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57187827"/>
+        <c:axId val="52922887"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1667,7 +1700,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95604837"/>
+        <c:crossAx val="62129246"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1675,7 +1708,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95604837"/>
+        <c:axId val="62129246"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1717,7 +1750,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57187827"/>
+        <c:crossAx val="52922887"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1911,58 +1944,58 @@
                 <c:formatCode>"S/ "#,##0;[RED]"-S/ "#,##0;\-</c:formatCode>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
-                  <c:v>1688</c:v>
+                  <c:v>1120</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3008</c:v>
+                  <c:v>2000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7680</c:v>
+                  <c:v>4912</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11040</c:v>
+                  <c:v>6936</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15825</c:v>
+                  <c:v>9797</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>19827</c:v>
+                  <c:v>12182</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>25312</c:v>
+                  <c:v>15481</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>29418</c:v>
+                  <c:v>17976</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>33311</c:v>
+                  <c:v>20349</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>37064</c:v>
+                  <c:v>22624</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>39384</c:v>
+                  <c:v>24032</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>42056</c:v>
+                  <c:v>25696</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>43564</c:v>
+                  <c:v>26708</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>47284</c:v>
+                  <c:v>29404</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>49134</c:v>
+                  <c:v>30622</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>52750</c:v>
+                  <c:v>32862</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>57754</c:v>
+                  <c:v>36338</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>59754</c:v>
+                  <c:v>37538</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2091,58 +2124,58 @@
                 <c:formatCode>"S/ "#,##0;[RED]"-S/ "#,##0;\-</c:formatCode>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>62279</c:v>
+                  <c:v>40063</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2271,58 +2304,58 @@
                 <c:formatCode>"S/ "#,##0;[RED]"-S/ "#,##0;\-</c:formatCode>
                 <c:ptCount val="18"/>
                 <c:pt idx="0">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>65393</c:v>
+                  <c:v>42066</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2337,11 +2370,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="71380727"/>
-        <c:axId val="77423519"/>
+        <c:axId val="60823393"/>
+        <c:axId val="77710426"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="71380727"/>
+        <c:axId val="60823393"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2373,7 +2406,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77423519"/>
+        <c:crossAx val="77710426"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2381,7 +2414,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77423519"/>
+        <c:axId val="77710426"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2457,7 +2490,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71380727"/>
+        <c:crossAx val="60823393"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2530,7 +2563,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="6673320" y="571680"/>
+        <a:off x="6955200" y="571680"/>
         <a:ext cx="6479640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2759,7 +2792,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -2794,7 +2827,7 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">Paquetes!M42</f>
-        <v>57152</v>
+        <v>35096</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>6</v>
@@ -2818,7 +2851,7 @@
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">Paquetes!V42-Paquetes!O42</f>
-        <v>392</v>
+        <v>232</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>10</v>
@@ -2830,7 +2863,7 @@
       </c>
       <c r="B8" s="7" t="n">
         <f aca="false">Presupuesto!B13</f>
-        <v>59754</v>
+        <v>37538</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>12</v>
@@ -2854,7 +2887,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">Presupuesto!B15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>16</v>
@@ -2866,7 +2899,7 @@
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">Presupuesto!B17</f>
-        <v>3114</v>
+        <v>2003</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>18</v>
@@ -2878,35 +2911,43 @@
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">Presupuesto!B18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>20</v>
       </c>
     </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <f aca="false">Presupuesto!B20</f>
+        <v>42200</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B15" s="13" t="s">
+      <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
+      <c r="B14" s="5" t="n">
+        <f aca="false">Presupuesto!B21</f>
+        <v>134</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="13" t="s">
+      <c r="A16" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="12" t="s">
         <v>26</v>
       </c>
       <c r="B17" s="13" t="s">
@@ -2914,31 +2955,31 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="14" t="s">
         <v>28</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>29</v>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>31</v>
+      </c>
+    </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="13" t="s">
+      <c r="A20" s="16" t="s">
         <v>32</v>
       </c>
+      <c r="B20" s="13" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="13" t="s">
+      <c r="A22" s="11" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2988,6 +3029,22 @@
       </c>
       <c r="B28" s="13" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -3019,17 +3076,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C4" s="18" t="n">
         <v>160</v>
@@ -3037,40 +3094,40 @@
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C7" s="19" t="n">
-        <v>8000</v>
+        <v>4800</v>
       </c>
       <c r="D7" s="20" t="n">
         <f aca="false">C7/$C$4</f>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E7" s="21" t="n">
         <f aca="false">Paquetes!D42</f>
@@ -3078,26 +3135,26 @@
       </c>
       <c r="F7" s="22" t="n">
         <f aca="false">D7*E7</f>
-        <v>15280</v>
+        <v>9168</v>
       </c>
       <c r="G7" s="23" t="n">
         <f aca="false">IF($F$15=0,0,F7/$F$15)</f>
-        <v>0.267357222844345</v>
+        <v>0.261226350581263</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>4960</v>
+        <v>3200</v>
       </c>
       <c r="D8" s="20" t="n">
         <f aca="false">C8/$C$4</f>
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="E8" s="21" t="n">
         <f aca="false">Paquetes!E42</f>
@@ -3105,26 +3162,26 @@
       </c>
       <c r="F8" s="22" t="n">
         <f aca="false">D8*E8</f>
-        <v>3968</v>
+        <v>2560</v>
       </c>
       <c r="G8" s="23" t="n">
         <f aca="false">IF($F$15=0,0,F8/$F$15)</f>
-        <v>0.0694288913773796</v>
+        <v>0.0729427855026214</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>7040</v>
+        <v>4000</v>
       </c>
       <c r="D9" s="20" t="n">
         <f aca="false">C9/$C$4</f>
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="E9" s="21" t="n">
         <f aca="false">Paquetes!F42</f>
@@ -3132,26 +3189,26 @@
       </c>
       <c r="F9" s="22" t="n">
         <f aca="false">D9*E9</f>
-        <v>9152</v>
+        <v>5200</v>
       </c>
       <c r="G9" s="23" t="n">
         <f aca="false">IF($F$15=0,0,F9/$F$15)</f>
-        <v>0.16013437849944</v>
+        <v>0.1481650330522</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C10" s="19" t="n">
-        <v>5600</v>
+        <v>3520</v>
       </c>
       <c r="D10" s="20" t="n">
         <f aca="false">C10/$C$4</f>
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="E10" s="21" t="n">
         <f aca="false">Paquetes!G42</f>
@@ -3159,26 +3216,26 @@
       </c>
       <c r="F10" s="22" t="n">
         <f aca="false">D10*E10</f>
-        <v>12040</v>
+        <v>7568</v>
       </c>
       <c r="G10" s="23" t="n">
         <f aca="false">IF($F$15=0,0,F10/$F$15)</f>
-        <v>0.210666293393057</v>
+        <v>0.215637109642124</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C11" s="19" t="n">
-        <v>5280</v>
+        <v>3200</v>
       </c>
       <c r="D11" s="20" t="n">
         <f aca="false">C11/$C$4</f>
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">Paquetes!H42</f>
@@ -3186,26 +3243,26 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">D11*E11</f>
-        <v>10032</v>
+        <v>6080</v>
       </c>
       <c r="G11" s="23" t="n">
         <f aca="false">IF($F$15=0,0,F11/$F$15)</f>
-        <v>0.175531914893617</v>
+        <v>0.173239115568726</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>4000</v>
+        <v>2560</v>
       </c>
       <c r="D12" s="20" t="n">
         <f aca="false">C12/$C$4</f>
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E12" s="21" t="n">
         <f aca="false">Paquetes!I42</f>
@@ -3213,19 +3270,19 @@
       </c>
       <c r="F12" s="22" t="n">
         <f aca="false">D12*E12</f>
-        <v>6000</v>
+        <v>3840</v>
       </c>
       <c r="G12" s="23" t="n">
         <f aca="false">IF($F$15=0,0,F12/$F$15)</f>
-        <v>0.10498320268757</v>
+        <v>0.109414178253932</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C13" s="19" t="n">
         <v>2400</v>
@@ -3244,15 +3301,15 @@
       </c>
       <c r="G13" s="23" t="n">
         <f aca="false">IF($F$15=0,0,F13/$F$15)</f>
-        <v>0.0083986562150056</v>
+        <v>0.0136767722817415</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C14" s="19" t="n">
         <v>4000</v>
@@ -3271,12 +3328,12 @@
       </c>
       <c r="G14" s="23" t="n">
         <f aca="false">IF($F$15=0,0,F14/$F$15)</f>
-        <v>0.00349944008958567</v>
+        <v>0.0056986551173923</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="24" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B15" s="25"/>
       <c r="C15" s="25"/>
@@ -3287,7 +3344,7 @@
       </c>
       <c r="F15" s="27" t="n">
         <f aca="false">SUM(F7:F14)</f>
-        <v>57152</v>
+        <v>35096</v>
       </c>
       <c r="G15" s="28" t="n">
         <f aca="false">SUM(G7:G14)</f>
@@ -3296,7 +3353,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -3331,15 +3388,15 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>3</v>
@@ -3347,10 +3404,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C5" s="19" t="n">
         <v>120</v>
@@ -3358,10 +3415,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C6" s="19" t="n">
         <v>480</v>
@@ -3369,10 +3426,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C7" s="19" t="n">
         <v>80</v>
@@ -3380,10 +3437,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C8" s="19" t="n">
         <v>380</v>
@@ -3391,10 +3448,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C9" s="19" t="n">
         <v>260</v>
@@ -3402,10 +3459,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C10" s="19" t="n">
         <v>180</v>
@@ -3413,10 +3470,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C11" s="19" t="n">
         <v>210</v>
@@ -3424,10 +3481,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C12" s="19" t="n">
         <v>500</v>
@@ -3435,7 +3492,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="24" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B13" s="25"/>
       <c r="C13" s="27" t="n">
@@ -3445,7 +3502,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -3477,41 +3534,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C4" s="29" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D4" s="30" t="n">
         <f aca="false">Tarifas!D7</f>
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E4" s="30" t="n">
         <f aca="false">Tarifas!D8</f>
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F4" s="30" t="n">
         <f aca="false">Tarifas!D9</f>
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="G4" s="30" t="n">
         <f aca="false">Tarifas!D10</f>
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="H4" s="30" t="n">
         <f aca="false">Tarifas!D11</f>
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="I4" s="30" t="n">
         <f aca="false">Tarifas!D12</f>
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="J4" s="30" t="n">
         <f aca="false">Tarifas!D13</f>
@@ -3524,81 +3581,81 @@
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="U5" s="3" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="V5" s="3" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D6" s="31" t="n">
         <v>24</v>
@@ -3616,7 +3673,7 @@
       </c>
       <c r="M6" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D6:K6,$D$4:$K$4),0)</f>
-        <v>1200</v>
+        <v>720</v>
       </c>
       <c r="N6" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A6,'No laborales'!$C$5:$C$12)</f>
@@ -3624,7 +3681,7 @@
       </c>
       <c r="O6" s="22" t="n">
         <f aca="false">M6+N6</f>
-        <v>1320</v>
+        <v>840</v>
       </c>
       <c r="P6" s="33"/>
       <c r="Q6" s="33"/>
@@ -3646,18 +3703,18 @@
       </c>
       <c r="V6" s="34" t="n">
         <f aca="false">IF(P6="",O6,ROUND(T6,0))</f>
-        <v>1320</v>
+        <v>840</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D7" s="31" t="n">
         <v>32</v>
@@ -3675,7 +3732,7 @@
       </c>
       <c r="M7" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D7:K7,$D$4:$K$4),0)</f>
-        <v>1600</v>
+        <v>960</v>
       </c>
       <c r="N7" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A7,'No laborales'!$C$5:$C$12)</f>
@@ -3683,7 +3740,7 @@
       </c>
       <c r="O7" s="22" t="n">
         <f aca="false">M7+N7</f>
-        <v>1600</v>
+        <v>960</v>
       </c>
       <c r="P7" s="33"/>
       <c r="Q7" s="33"/>
@@ -3705,18 +3762,18 @@
       </c>
       <c r="V7" s="34" t="n">
         <f aca="false">IF(P7="",O7,ROUND(T7,0))</f>
-        <v>1600</v>
+        <v>960</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D8" s="31" t="n">
         <v>201.6</v>
@@ -3734,7 +3791,7 @@
       </c>
       <c r="M8" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D8:K8,$D$4:$K$4),0)</f>
-        <v>10080</v>
+        <v>6048</v>
       </c>
       <c r="N8" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A8,'No laborales'!$C$5:$C$12)</f>
@@ -3742,7 +3799,7 @@
       </c>
       <c r="O8" s="22" t="n">
         <f aca="false">M8+N8</f>
-        <v>10560</v>
+        <v>6528</v>
       </c>
       <c r="P8" s="33"/>
       <c r="Q8" s="33"/>
@@ -3764,18 +3821,18 @@
       </c>
       <c r="V8" s="34" t="n">
         <f aca="false">IF(P8="",O8,ROUND(T8,0))</f>
-        <v>10560</v>
+        <v>6528</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D9" s="31" t="n">
         <v>24</v>
@@ -3793,7 +3850,7 @@
       </c>
       <c r="M9" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D9:K9,$D$4:$K$4),0)</f>
-        <v>1200</v>
+        <v>720</v>
       </c>
       <c r="N9" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A9,'No laborales'!$C$5:$C$12)</f>
@@ -3801,7 +3858,7 @@
       </c>
       <c r="O9" s="22" t="n">
         <f aca="false">M9+N9</f>
-        <v>1200</v>
+        <v>720</v>
       </c>
       <c r="P9" s="33"/>
       <c r="Q9" s="33"/>
@@ -3823,18 +3880,18 @@
       </c>
       <c r="V9" s="34" t="n">
         <f aca="false">IF(P9="",O9,ROUND(T9,0))</f>
-        <v>1200</v>
+        <v>720</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D10" s="31"/>
       <c r="E10" s="31" t="n">
@@ -3854,7 +3911,7 @@
       </c>
       <c r="M10" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D10:K10,$D$4:$K$4),0)</f>
-        <v>1112</v>
+        <v>760</v>
       </c>
       <c r="N10" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A10,'No laborales'!$C$5:$C$12)</f>
@@ -3862,7 +3919,7 @@
       </c>
       <c r="O10" s="22" t="n">
         <f aca="false">M10+N10</f>
-        <v>1192</v>
+        <v>840</v>
       </c>
       <c r="P10" s="33"/>
       <c r="Q10" s="33"/>
@@ -3884,18 +3941,18 @@
       </c>
       <c r="V10" s="34" t="n">
         <f aca="false">IF(P10="",O10,ROUND(T10,0))</f>
-        <v>1192</v>
+        <v>840</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D11" s="31"/>
       <c r="E11" s="31" t="n">
@@ -3913,7 +3970,7 @@
       </c>
       <c r="M11" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D11:K11,$D$4:$K$4),0)</f>
-        <v>992</v>
+        <v>640</v>
       </c>
       <c r="N11" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A11,'No laborales'!$C$5:$C$12)</f>
@@ -3921,7 +3978,7 @@
       </c>
       <c r="O11" s="22" t="n">
         <f aca="false">M11+N11</f>
-        <v>992</v>
+        <v>640</v>
       </c>
       <c r="P11" s="33"/>
       <c r="Q11" s="33"/>
@@ -3943,18 +4000,18 @@
       </c>
       <c r="V11" s="34" t="n">
         <f aca="false">IF(P11="",O11,ROUND(T11,0))</f>
-        <v>992</v>
+        <v>640</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>125</v>
-      </c>
       <c r="C12" s="4" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D12" s="31"/>
       <c r="E12" s="31"/>
@@ -3972,7 +4029,7 @@
       </c>
       <c r="M12" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D12:K12,$D$4:$K$4),0)</f>
-        <v>1120</v>
+        <v>704</v>
       </c>
       <c r="N12" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A12,'No laborales'!$C$5:$C$12)</f>
@@ -3980,7 +4037,7 @@
       </c>
       <c r="O12" s="22" t="n">
         <f aca="false">M12+N12</f>
-        <v>1120</v>
+        <v>704</v>
       </c>
       <c r="P12" s="33"/>
       <c r="Q12" s="33"/>
@@ -4002,18 +4059,18 @@
       </c>
       <c r="V12" s="34" t="n">
         <f aca="false">IF(P12="",O12,ROUND(T12,0))</f>
-        <v>1120</v>
+        <v>704</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D13" s="31"/>
       <c r="E13" s="31"/>
@@ -4031,7 +4088,7 @@
       </c>
       <c r="M13" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D13:K13,$D$4:$K$4),0)</f>
-        <v>1056</v>
+        <v>640</v>
       </c>
       <c r="N13" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A13,'No laborales'!$C$5:$C$12)</f>
@@ -4039,7 +4096,7 @@
       </c>
       <c r="O13" s="22" t="n">
         <f aca="false">M13+N13</f>
-        <v>1056</v>
+        <v>640</v>
       </c>
       <c r="P13" s="33"/>
       <c r="Q13" s="33"/>
@@ -4061,18 +4118,18 @@
       </c>
       <c r="V13" s="34" t="n">
         <f aca="false">IF(P13="",O13,ROUND(T13,0))</f>
-        <v>1056</v>
+        <v>640</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D14" s="31"/>
       <c r="E14" s="31" t="n">
@@ -4090,7 +4147,7 @@
       </c>
       <c r="M14" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D14:K14,$D$4:$K$4),0)</f>
-        <v>744</v>
+        <v>480</v>
       </c>
       <c r="N14" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A14,'No laborales'!$C$5:$C$12)</f>
@@ -4098,7 +4155,7 @@
       </c>
       <c r="O14" s="22" t="n">
         <f aca="false">M14+N14</f>
-        <v>744</v>
+        <v>480</v>
       </c>
       <c r="P14" s="33"/>
       <c r="Q14" s="33"/>
@@ -4120,18 +4177,18 @@
       </c>
       <c r="V14" s="34" t="n">
         <f aca="false">IF(P14="",O14,ROUND(T14,0))</f>
-        <v>744</v>
+        <v>480</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D15" s="31"/>
       <c r="E15" s="31"/>
@@ -4149,7 +4206,7 @@
       </c>
       <c r="M15" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D15:K15,$D$4:$K$4),0)</f>
-        <v>1056</v>
+        <v>600</v>
       </c>
       <c r="N15" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A15,'No laborales'!$C$5:$C$12)</f>
@@ -4157,7 +4214,7 @@
       </c>
       <c r="O15" s="22" t="n">
         <f aca="false">M15+N15</f>
-        <v>1056</v>
+        <v>600</v>
       </c>
       <c r="P15" s="33"/>
       <c r="Q15" s="33"/>
@@ -4179,18 +4236,18 @@
       </c>
       <c r="V15" s="34" t="n">
         <f aca="false">IF(P15="",O15,ROUND(T15,0))</f>
-        <v>1056</v>
+        <v>600</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D16" s="31"/>
       <c r="E16" s="31"/>
@@ -4208,7 +4265,7 @@
       </c>
       <c r="M16" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D16:K16,$D$4:$K$4),0)</f>
-        <v>1408</v>
+        <v>800</v>
       </c>
       <c r="N16" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A16,'No laborales'!$C$5:$C$12)</f>
@@ -4216,7 +4273,7 @@
       </c>
       <c r="O16" s="22" t="n">
         <f aca="false">M16+N16</f>
-        <v>1408</v>
+        <v>800</v>
       </c>
       <c r="P16" s="33"/>
       <c r="Q16" s="33"/>
@@ -4238,18 +4295,18 @@
       </c>
       <c r="V16" s="34" t="n">
         <f aca="false">IF(P16="",O16,ROUND(T16,0))</f>
-        <v>1408</v>
+        <v>800</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>136</v>
-      </c>
       <c r="C17" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D17" s="31"/>
       <c r="E17" s="31"/>
@@ -4267,7 +4324,7 @@
       </c>
       <c r="M17" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D17:K17,$D$4:$K$4),0)</f>
-        <v>1760</v>
+        <v>1000</v>
       </c>
       <c r="N17" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A17,'No laborales'!$C$5:$C$12)</f>
@@ -4275,7 +4332,7 @@
       </c>
       <c r="O17" s="22" t="n">
         <f aca="false">M17+N17</f>
-        <v>1760</v>
+        <v>1000</v>
       </c>
       <c r="P17" s="33"/>
       <c r="Q17" s="33"/>
@@ -4297,18 +4354,18 @@
       </c>
       <c r="V17" s="34" t="n">
         <f aca="false">IF(P17="",O17,ROUND(T17,0))</f>
-        <v>1760</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D18" s="31"/>
       <c r="E18" s="31"/>
@@ -4326,7 +4383,7 @@
       </c>
       <c r="M18" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D18:K18,$D$4:$K$4),0)</f>
-        <v>2464</v>
+        <v>1400</v>
       </c>
       <c r="N18" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A18,'No laborales'!$C$5:$C$12)</f>
@@ -4334,7 +4391,7 @@
       </c>
       <c r="O18" s="22" t="n">
         <f aca="false">M18+N18</f>
-        <v>2464</v>
+        <v>1400</v>
       </c>
       <c r="P18" s="35" t="n">
         <v>0.85</v>
@@ -4344,34 +4401,34 @@
       </c>
       <c r="R18" s="22" t="n">
         <f aca="false">IF(P18="","",O18*P18)</f>
-        <v>2094.4</v>
+        <v>1190</v>
       </c>
       <c r="S18" s="22" t="n">
         <f aca="false">IF(Q18="","",O18*Q18)</f>
-        <v>3942.4</v>
+        <v>2240</v>
       </c>
       <c r="T18" s="22" t="n">
         <f aca="false">IF(P18="","",(R18+4*O18+S18)/6)</f>
-        <v>2648.8</v>
+        <v>1505</v>
       </c>
       <c r="U18" s="22" t="n">
         <f aca="false">IF(P18="","",(S18-R18)/6)</f>
-        <v>308</v>
+        <v>175</v>
       </c>
       <c r="V18" s="34" t="n">
         <f aca="false">IF(P18="",O18,ROUND(T18,0))</f>
-        <v>2649</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D19" s="31"/>
       <c r="E19" s="31"/>
@@ -4391,7 +4448,7 @@
       </c>
       <c r="M19" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D19:K19,$D$4:$K$4),0)</f>
-        <v>1608</v>
+        <v>1000</v>
       </c>
       <c r="N19" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A19,'No laborales'!$C$5:$C$12)</f>
@@ -4399,7 +4456,7 @@
       </c>
       <c r="O19" s="22" t="n">
         <f aca="false">M19+N19</f>
-        <v>1608</v>
+        <v>1000</v>
       </c>
       <c r="P19" s="33"/>
       <c r="Q19" s="33"/>
@@ -4421,18 +4478,18 @@
       </c>
       <c r="V19" s="34" t="n">
         <f aca="false">IF(P19="",O19,ROUND(T19,0))</f>
-        <v>1608</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D20" s="31"/>
       <c r="E20" s="31"/>
@@ -4450,7 +4507,7 @@
       </c>
       <c r="M20" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D20:K20,$D$4:$K$4),0)</f>
-        <v>840</v>
+        <v>528</v>
       </c>
       <c r="N20" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A20,'No laborales'!$C$5:$C$12)</f>
@@ -4458,7 +4515,7 @@
       </c>
       <c r="O20" s="22" t="n">
         <f aca="false">M20+N20</f>
-        <v>840</v>
+        <v>528</v>
       </c>
       <c r="P20" s="33"/>
       <c r="Q20" s="33"/>
@@ -4480,18 +4537,18 @@
       </c>
       <c r="V20" s="34" t="n">
         <f aca="false">IF(P20="",O20,ROUND(T20,0))</f>
-        <v>840</v>
+        <v>528</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D21" s="31"/>
       <c r="E21" s="31"/>
@@ -4509,7 +4566,7 @@
       </c>
       <c r="M21" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D21:K21,$D$4:$K$4),0)</f>
-        <v>840</v>
+        <v>528</v>
       </c>
       <c r="N21" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A21,'No laborales'!$C$5:$C$12)</f>
@@ -4517,7 +4574,7 @@
       </c>
       <c r="O21" s="22" t="n">
         <f aca="false">M21+N21</f>
-        <v>840</v>
+        <v>528</v>
       </c>
       <c r="P21" s="33"/>
       <c r="Q21" s="33"/>
@@ -4539,18 +4596,18 @@
       </c>
       <c r="V21" s="34" t="n">
         <f aca="false">IF(P21="",O21,ROUND(T21,0))</f>
-        <v>840</v>
+        <v>528</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>147</v>
-      </c>
       <c r="C22" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D22" s="31"/>
       <c r="E22" s="31"/>
@@ -4568,7 +4625,7 @@
       </c>
       <c r="M22" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D22:K22,$D$4:$K$4),0)</f>
-        <v>840</v>
+        <v>528</v>
       </c>
       <c r="N22" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A22,'No laborales'!$C$5:$C$12)</f>
@@ -4576,7 +4633,7 @@
       </c>
       <c r="O22" s="22" t="n">
         <f aca="false">M22+N22</f>
-        <v>840</v>
+        <v>528</v>
       </c>
       <c r="P22" s="35" t="n">
         <v>0.85</v>
@@ -4586,34 +4643,34 @@
       </c>
       <c r="R22" s="22" t="n">
         <f aca="false">IF(P22="","",O22*P22)</f>
-        <v>714</v>
+        <v>448.8</v>
       </c>
       <c r="S22" s="22" t="n">
         <f aca="false">IF(Q22="","",O22*Q22)</f>
-        <v>1260</v>
+        <v>792</v>
       </c>
       <c r="T22" s="22" t="n">
         <f aca="false">IF(P22="","",(R22+4*O22+S22)/6)</f>
-        <v>889</v>
+        <v>558.8</v>
       </c>
       <c r="U22" s="22" t="n">
         <f aca="false">IF(P22="","",(S22-R22)/6)</f>
-        <v>91</v>
+        <v>57.2</v>
       </c>
       <c r="V22" s="34" t="n">
         <f aca="false">IF(P22="",O22,ROUND(T22,0))</f>
-        <v>889</v>
+        <v>559</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D23" s="31"/>
       <c r="E23" s="31"/>
@@ -4633,7 +4690,7 @@
       </c>
       <c r="M23" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D23:K23,$D$4:$K$4),0)</f>
-        <v>1472</v>
+        <v>904</v>
       </c>
       <c r="N23" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A23,'No laborales'!$C$5:$C$12)</f>
@@ -4641,7 +4698,7 @@
       </c>
       <c r="O23" s="22" t="n">
         <f aca="false">M23+N23</f>
-        <v>1472</v>
+        <v>904</v>
       </c>
       <c r="P23" s="33"/>
       <c r="Q23" s="33"/>
@@ -4663,18 +4720,18 @@
       </c>
       <c r="V23" s="34" t="n">
         <f aca="false">IF(P23="",O23,ROUND(T23,0))</f>
-        <v>1472</v>
+        <v>904</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D24" s="31"/>
       <c r="E24" s="31"/>
@@ -4692,7 +4749,7 @@
       </c>
       <c r="M24" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D24:K24,$D$4:$K$4),0)</f>
-        <v>1680</v>
+        <v>1056</v>
       </c>
       <c r="N24" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A24,'No laborales'!$C$5:$C$12)</f>
@@ -4700,7 +4757,7 @@
       </c>
       <c r="O24" s="22" t="n">
         <f aca="false">M24+N24</f>
-        <v>1680</v>
+        <v>1056</v>
       </c>
       <c r="P24" s="33"/>
       <c r="Q24" s="33"/>
@@ -4722,18 +4779,18 @@
       </c>
       <c r="V24" s="34" t="n">
         <f aca="false">IF(P24="",O24,ROUND(T24,0))</f>
-        <v>1680</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D25" s="31"/>
       <c r="E25" s="31"/>
@@ -4751,7 +4808,7 @@
       </c>
       <c r="M25" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D25:K25,$D$4:$K$4),0)</f>
-        <v>792</v>
+        <v>480</v>
       </c>
       <c r="N25" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A25,'No laborales'!$C$5:$C$12)</f>
@@ -4759,7 +4816,7 @@
       </c>
       <c r="O25" s="22" t="n">
         <f aca="false">M25+N25</f>
-        <v>792</v>
+        <v>480</v>
       </c>
       <c r="P25" s="33"/>
       <c r="Q25" s="33"/>
@@ -4781,18 +4838,18 @@
       </c>
       <c r="V25" s="34" t="n">
         <f aca="false">IF(P25="",O25,ROUND(T25,0))</f>
-        <v>792</v>
+        <v>480</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D26" s="31"/>
       <c r="E26" s="31"/>
@@ -4810,7 +4867,7 @@
       </c>
       <c r="M26" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D26:K26,$D$4:$K$4),0)</f>
-        <v>1320</v>
+        <v>800</v>
       </c>
       <c r="N26" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A26,'No laborales'!$C$5:$C$12)</f>
@@ -4818,7 +4875,7 @@
       </c>
       <c r="O26" s="22" t="n">
         <f aca="false">M26+N26</f>
-        <v>1320</v>
+        <v>800</v>
       </c>
       <c r="P26" s="33"/>
       <c r="Q26" s="33"/>
@@ -4840,18 +4897,18 @@
       </c>
       <c r="V26" s="34" t="n">
         <f aca="false">IF(P26="",O26,ROUND(T26,0))</f>
-        <v>1320</v>
+        <v>800</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>158</v>
-      </c>
       <c r="C27" s="4" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D27" s="31"/>
       <c r="E27" s="31"/>
@@ -4869,7 +4926,7 @@
       </c>
       <c r="M27" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D27:K27,$D$4:$K$4),0)</f>
-        <v>1584</v>
+        <v>960</v>
       </c>
       <c r="N27" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A27,'No laborales'!$C$5:$C$12)</f>
@@ -4877,7 +4934,7 @@
       </c>
       <c r="O27" s="22" t="n">
         <f aca="false">M27+N27</f>
-        <v>1584</v>
+        <v>960</v>
       </c>
       <c r="P27" s="33"/>
       <c r="Q27" s="33"/>
@@ -4899,18 +4956,18 @@
       </c>
       <c r="V27" s="34" t="n">
         <f aca="false">IF(P27="",O27,ROUND(T27,0))</f>
-        <v>1584</v>
+        <v>960</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D28" s="31"/>
       <c r="E28" s="31"/>
@@ -4928,7 +4985,7 @@
       </c>
       <c r="M28" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D28:K28,$D$4:$K$4),0)</f>
-        <v>1056</v>
+        <v>640</v>
       </c>
       <c r="N28" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A28,'No laborales'!$C$5:$C$12)</f>
@@ -4936,7 +4993,7 @@
       </c>
       <c r="O28" s="22" t="n">
         <f aca="false">M28+N28</f>
-        <v>1056</v>
+        <v>640</v>
       </c>
       <c r="P28" s="33"/>
       <c r="Q28" s="33"/>
@@ -4958,18 +5015,18 @@
       </c>
       <c r="V28" s="34" t="n">
         <f aca="false">IF(P28="",O28,ROUND(T28,0))</f>
-        <v>1056</v>
+        <v>640</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D29" s="31"/>
       <c r="E29" s="31"/>
@@ -4987,7 +5044,7 @@
       </c>
       <c r="M29" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D29:K29,$D$4:$K$4),0)</f>
-        <v>840</v>
+        <v>528</v>
       </c>
       <c r="N29" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A29,'No laborales'!$C$5:$C$12)</f>
@@ -4995,7 +5052,7 @@
       </c>
       <c r="O29" s="22" t="n">
         <f aca="false">M29+N29</f>
-        <v>840</v>
+        <v>528</v>
       </c>
       <c r="P29" s="33"/>
       <c r="Q29" s="33"/>
@@ -5017,18 +5074,18 @@
       </c>
       <c r="V29" s="34" t="n">
         <f aca="false">IF(P29="",O29,ROUND(T29,0))</f>
-        <v>840</v>
+        <v>528</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="D30" s="31"/>
       <c r="E30" s="31"/>
@@ -5048,7 +5105,7 @@
       </c>
       <c r="M30" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D30:K30,$D$4:$K$4),0)</f>
-        <v>2104</v>
+        <v>1280</v>
       </c>
       <c r="N30" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A30,'No laborales'!$C$5:$C$12)</f>
@@ -5056,7 +5113,7 @@
       </c>
       <c r="O30" s="22" t="n">
         <f aca="false">M30+N30</f>
-        <v>2104</v>
+        <v>1280</v>
       </c>
       <c r="P30" s="35" t="n">
         <v>0.85</v>
@@ -5066,34 +5123,34 @@
       </c>
       <c r="R30" s="22" t="n">
         <f aca="false">IF(P30="","",O30*P30)</f>
-        <v>1788.4</v>
+        <v>1088</v>
       </c>
       <c r="S30" s="22" t="n">
         <f aca="false">IF(Q30="","",O30*Q30)</f>
-        <v>3366.4</v>
+        <v>2048</v>
       </c>
       <c r="T30" s="22" t="n">
         <f aca="false">IF(P30="","",(R30+4*O30+S30)/6)</f>
-        <v>2261.8</v>
+        <v>1376</v>
       </c>
       <c r="U30" s="22" t="n">
         <f aca="false">IF(P30="","",(S30-R30)/6)</f>
-        <v>263</v>
+        <v>160</v>
       </c>
       <c r="V30" s="34" t="n">
         <f aca="false">IF(P30="",O30,ROUND(T30,0))</f>
-        <v>2262</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>167</v>
-      </c>
       <c r="C31" s="4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="D31" s="31"/>
       <c r="E31" s="31"/>
@@ -5111,7 +5168,7 @@
       </c>
       <c r="M31" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D31:K31,$D$4:$K$4),0)</f>
-        <v>1320</v>
+        <v>800</v>
       </c>
       <c r="N31" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A31,'No laborales'!$C$5:$C$12)</f>
@@ -5119,7 +5176,7 @@
       </c>
       <c r="O31" s="22" t="n">
         <f aca="false">M31+N31</f>
-        <v>1320</v>
+        <v>800</v>
       </c>
       <c r="P31" s="33"/>
       <c r="Q31" s="33"/>
@@ -5141,18 +5198,18 @@
       </c>
       <c r="V31" s="34" t="n">
         <f aca="false">IF(P31="",O31,ROUND(T31,0))</f>
-        <v>1320</v>
+        <v>800</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D32" s="31"/>
       <c r="E32" s="31"/>
@@ -5170,7 +5227,7 @@
       </c>
       <c r="M32" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D32:K32,$D$4:$K$4),0)</f>
-        <v>792</v>
+        <v>480</v>
       </c>
       <c r="N32" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A32,'No laborales'!$C$5:$C$12)</f>
@@ -5178,7 +5235,7 @@
       </c>
       <c r="O32" s="22" t="n">
         <f aca="false">M32+N32</f>
-        <v>792</v>
+        <v>480</v>
       </c>
       <c r="P32" s="33"/>
       <c r="Q32" s="33"/>
@@ -5200,18 +5257,18 @@
       </c>
       <c r="V32" s="34" t="n">
         <f aca="false">IF(P32="",O32,ROUND(T32,0))</f>
-        <v>792</v>
+        <v>480</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D33" s="31"/>
       <c r="E33" s="31"/>
@@ -5229,7 +5286,7 @@
       </c>
       <c r="M33" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D33:K33,$D$4:$K$4),0)</f>
-        <v>800</v>
+        <v>512</v>
       </c>
       <c r="N33" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A33,'No laborales'!$C$5:$C$12)</f>
@@ -5237,7 +5294,7 @@
       </c>
       <c r="O33" s="22" t="n">
         <f aca="false">M33+N33</f>
-        <v>800</v>
+        <v>512</v>
       </c>
       <c r="P33" s="33"/>
       <c r="Q33" s="33"/>
@@ -5259,18 +5316,18 @@
       </c>
       <c r="V33" s="34" t="n">
         <f aca="false">IF(P33="",O33,ROUND(T33,0))</f>
-        <v>800</v>
+        <v>512</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D34" s="31"/>
       <c r="E34" s="31"/>
@@ -5288,7 +5345,7 @@
       </c>
       <c r="M34" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D34:K34,$D$4:$K$4),0)</f>
-        <v>1400</v>
+        <v>896</v>
       </c>
       <c r="N34" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A34,'No laborales'!$C$5:$C$12)</f>
@@ -5296,7 +5353,7 @@
       </c>
       <c r="O34" s="22" t="n">
         <f aca="false">M34+N34</f>
-        <v>1400</v>
+        <v>896</v>
       </c>
       <c r="P34" s="33"/>
       <c r="Q34" s="33"/>
@@ -5318,18 +5375,18 @@
       </c>
       <c r="V34" s="34" t="n">
         <f aca="false">IF(P34="",O34,ROUND(T34,0))</f>
-        <v>1400</v>
+        <v>896</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>176</v>
-      </c>
       <c r="C35" s="4" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="D35" s="31"/>
       <c r="E35" s="31"/>
@@ -5347,7 +5404,7 @@
       </c>
       <c r="M35" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D35:K35,$D$4:$K$4),0)</f>
-        <v>800</v>
+        <v>512</v>
       </c>
       <c r="N35" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A35,'No laborales'!$C$5:$C$12)</f>
@@ -5355,7 +5412,7 @@
       </c>
       <c r="O35" s="22" t="n">
         <f aca="false">M35+N35</f>
-        <v>800</v>
+        <v>512</v>
       </c>
       <c r="P35" s="33"/>
       <c r="Q35" s="33"/>
@@ -5377,18 +5434,18 @@
       </c>
       <c r="V35" s="34" t="n">
         <f aca="false">IF(P35="",O35,ROUND(T35,0))</f>
-        <v>800</v>
+        <v>512</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D36" s="31"/>
       <c r="E36" s="31"/>
@@ -5408,7 +5465,7 @@
       </c>
       <c r="M36" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D36:K36,$D$4:$K$4),0)</f>
-        <v>840</v>
+        <v>624</v>
       </c>
       <c r="N36" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A36,'No laborales'!$C$5:$C$12)</f>
@@ -5416,7 +5473,7 @@
       </c>
       <c r="O36" s="22" t="n">
         <f aca="false">M36+N36</f>
-        <v>840</v>
+        <v>624</v>
       </c>
       <c r="P36" s="33"/>
       <c r="Q36" s="33"/>
@@ -5438,18 +5495,18 @@
       </c>
       <c r="V36" s="34" t="n">
         <f aca="false">IF(P36="",O36,ROUND(T36,0))</f>
-        <v>840</v>
+        <v>624</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D37" s="31"/>
       <c r="E37" s="31"/>
@@ -5467,7 +5524,7 @@
       </c>
       <c r="M37" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D37:K37,$D$4:$K$4),0)</f>
-        <v>1120</v>
+        <v>704</v>
       </c>
       <c r="N37" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A37,'No laborales'!$C$5:$C$12)</f>
@@ -5475,7 +5532,7 @@
       </c>
       <c r="O37" s="22" t="n">
         <f aca="false">M37+N37</f>
-        <v>1760</v>
+        <v>1344</v>
       </c>
       <c r="P37" s="33"/>
       <c r="Q37" s="33"/>
@@ -5497,18 +5554,18 @@
       </c>
       <c r="V37" s="34" t="n">
         <f aca="false">IF(P37="",O37,ROUND(T37,0))</f>
-        <v>1760</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D38" s="31"/>
       <c r="E38" s="31" t="n">
@@ -5526,7 +5583,7 @@
       </c>
       <c r="M38" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D38:K38,$D$4:$K$4),0)</f>
-        <v>992</v>
+        <v>640</v>
       </c>
       <c r="N38" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A38,'No laborales'!$C$5:$C$12)</f>
@@ -5534,7 +5591,7 @@
       </c>
       <c r="O38" s="22" t="n">
         <f aca="false">M38+N38</f>
-        <v>1172</v>
+        <v>820</v>
       </c>
       <c r="P38" s="33"/>
       <c r="Q38" s="33"/>
@@ -5556,18 +5613,18 @@
       </c>
       <c r="V38" s="34" t="n">
         <f aca="false">IF(P38="",O38,ROUND(T38,0))</f>
-        <v>1172</v>
+        <v>820</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D39" s="31"/>
       <c r="E39" s="31"/>
@@ -5587,7 +5644,7 @@
       </c>
       <c r="M39" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D39:K39,$D$4:$K$4),0)</f>
-        <v>920</v>
+        <v>632</v>
       </c>
       <c r="N39" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A39,'No laborales'!$C$5:$C$12)</f>
@@ -5595,7 +5652,7 @@
       </c>
       <c r="O39" s="22" t="n">
         <f aca="false">M39+N39</f>
-        <v>1130</v>
+        <v>842</v>
       </c>
       <c r="P39" s="33"/>
       <c r="Q39" s="33"/>
@@ -5617,18 +5674,18 @@
       </c>
       <c r="V39" s="34" t="n">
         <f aca="false">IF(P39="",O39,ROUND(T39,0))</f>
-        <v>1130</v>
+        <v>842</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D40" s="31" t="n">
         <v>8</v>
@@ -5654,7 +5711,7 @@
       </c>
       <c r="M40" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D40:K40,$D$4:$K$4),0)</f>
-        <v>6600</v>
+        <v>4112</v>
       </c>
       <c r="N40" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A40,'No laborales'!$C$5:$C$12)</f>
@@ -5662,7 +5719,7 @@
       </c>
       <c r="O40" s="22" t="n">
         <f aca="false">M40+N40</f>
-        <v>7100</v>
+        <v>4612</v>
       </c>
       <c r="P40" s="33"/>
       <c r="Q40" s="33"/>
@@ -5684,18 +5741,18 @@
       </c>
       <c r="V40" s="34" t="n">
         <f aca="false">IF(P40="",O40,ROUND(T40,0))</f>
-        <v>7100</v>
+        <v>4612</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D41" s="31" t="n">
         <v>16</v>
@@ -5713,7 +5770,7 @@
       </c>
       <c r="M41" s="22" t="n">
         <f aca="false">ROUND(SUMPRODUCT(D41:K41,$D$4:$K$4),0)</f>
-        <v>800</v>
+        <v>480</v>
       </c>
       <c r="N41" s="5" t="n">
         <f aca="false">SUMIF('No laborales'!$A$5:$A$12,A41,'No laborales'!$C$5:$C$12)</f>
@@ -5721,7 +5778,7 @@
       </c>
       <c r="O41" s="22" t="n">
         <f aca="false">M41+N41</f>
-        <v>800</v>
+        <v>480</v>
       </c>
       <c r="P41" s="33"/>
       <c r="Q41" s="33"/>
@@ -5743,12 +5800,12 @@
       </c>
       <c r="V41" s="34" t="n">
         <f aca="false">IF(P41="",O41,ROUND(T41,0))</f>
-        <v>800</v>
+        <v>480</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B42" s="25"/>
       <c r="C42" s="25"/>
@@ -5790,7 +5847,7 @@
       </c>
       <c r="M42" s="27" t="n">
         <f aca="false">SUM(M6:M41)</f>
-        <v>57152</v>
+        <v>35096</v>
       </c>
       <c r="N42" s="27" t="n">
         <f aca="false">SUM(N6:N41)</f>
@@ -5798,7 +5855,7 @@
       </c>
       <c r="O42" s="27" t="n">
         <f aca="false">SUM(O6:O41)</f>
-        <v>59362</v>
+        <v>37306</v>
       </c>
       <c r="P42" s="25"/>
       <c r="Q42" s="25"/>
@@ -5808,12 +5865,12 @@
       <c r="U42" s="25"/>
       <c r="V42" s="27" t="n">
         <f aca="false">SUM(V6:V41)</f>
-        <v>59754</v>
+        <v>37538</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -5843,37 +5900,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C5" s="36" t="n">
         <v>0.4</v>
@@ -5888,10 +5945,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C6" s="36" t="n">
         <v>0.3</v>
@@ -5906,10 +5963,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>0.25</v>
@@ -5924,10 +5981,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C8" s="36" t="n">
         <v>0.35</v>
@@ -5942,10 +5999,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C9" s="36" t="n">
         <v>0.1</v>
@@ -5972,7 +6029,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -5991,137 +6048,137 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">SUMIF(Paquetes!$B$6:$B$41,A5,Paquetes!$V$6:$V$41)</f>
-        <v>14680</v>
+        <v>9048</v>
       </c>
       <c r="C5" s="23" t="n">
         <f aca="false">IF($B$13=0,0,B5/$B$13)</f>
-        <v>0.24567392977876</v>
+        <v>0.241035750439555</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">SUMIF(Paquetes!$B$6:$B$41,A6,Paquetes!$V$6:$V$41)</f>
-        <v>5104</v>
+        <v>3304</v>
       </c>
       <c r="C6" s="23" t="n">
         <f aca="false">IF($B$13=0,0,B6/$B$13)</f>
-        <v>0.0854168758576832</v>
+        <v>0.0880174756247003</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">SUMIF(Paquetes!$B$6:$B$41,A7,Paquetes!$V$6:$V$41)</f>
-        <v>8481</v>
+        <v>4905</v>
       </c>
       <c r="C7" s="23" t="n">
         <f aca="false">IF($B$13=0,0,B7/$B$13)</f>
-        <v>0.14193192087559</v>
+        <v>0.130667590175289</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMIF(Paquetes!$B$6:$B$41,A8,Paquetes!$V$6:$V$41)</f>
-        <v>5721</v>
+        <v>3575</v>
       </c>
       <c r="C8" s="23" t="n">
         <f aca="false">IF($B$13=0,0,B8/$B$13)</f>
-        <v>0.0957425444321719</v>
+        <v>0.0952368266822953</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">SUMIF(Paquetes!$B$6:$B$41,A9,Paquetes!$V$6:$V$41)</f>
-        <v>4752</v>
+        <v>2880</v>
       </c>
       <c r="C9" s="23" t="n">
         <f aca="false">IF($B$13=0,0,B9/$B$13)</f>
-        <v>0.0795260568330154</v>
+        <v>0.0767222547818211</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">SUMIF(Paquetes!$B$6:$B$41,A10,Paquetes!$V$6:$V$41)</f>
-        <v>5214</v>
+        <v>3184</v>
       </c>
       <c r="C10" s="23" t="n">
         <f aca="false">IF($B$13=0,0,B10/$B$13)</f>
-        <v>0.0872577568028919</v>
+        <v>0.0848207150087911</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">SUMIF(Paquetes!$B$6:$B$41,A11,Paquetes!$V$6:$V$41)</f>
-        <v>3840</v>
+        <v>2544</v>
       </c>
       <c r="C11" s="23" t="n">
         <f aca="false">IF($B$13=0,0,B11/$B$13)</f>
-        <v>0.0642634802691033</v>
+        <v>0.0677713250572753</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B12" s="5" t="n">
         <f aca="false">SUMIF(Paquetes!$B$6:$B$41,A12,Paquetes!$V$6:$V$41)</f>
-        <v>11962</v>
+        <v>8098</v>
       </c>
       <c r="C12" s="23" t="n">
         <f aca="false">IF($B$13=0,0,B12/$B$13)</f>
-        <v>0.200187435150785</v>
+        <v>0.215728062230273</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6130,7 +6187,7 @@
       </c>
       <c r="B13" s="27" t="n">
         <f aca="false">SUM(B5:B12)</f>
-        <v>59754</v>
+        <v>37538</v>
       </c>
       <c r="C13" s="28" t="n">
         <f aca="false">SUM(C5:C12)</f>
@@ -6139,7 +6196,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B14" s="5" t="n">
         <f aca="false">Riesgos!E10</f>
@@ -6153,13 +6210,13 @@
       </c>
       <c r="B15" s="37" t="n">
         <f aca="false">B13+B14</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="C15" s="8"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B16" s="38" t="n">
         <v>0.05</v>
@@ -6168,11 +6225,11 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">ROUND(B15*B16,0)</f>
-        <v>3114</v>
+        <v>2003</v>
       </c>
       <c r="C17" s="4"/>
     </row>
@@ -6182,9 +6239,41 @@
       </c>
       <c r="B18" s="10" t="n">
         <f aca="false">B15+B17</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
       <c r="C18" s="39"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B20" s="40" t="n">
+        <v>42200</v>
+      </c>
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B21" s="22" t="n">
+        <f aca="false">B20-B18</f>
+        <v>134</v>
+      </c>
+      <c r="C21" s="4" t="str">
+        <f aca="false">IF(B21&gt;=0,"Dentro de lo autorizado","Excede lo autorizado")</f>
+        <v>Dentro de lo autorizado</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B22" s="22" t="n">
+        <f aca="false">B20*1.1</f>
+        <v>46420</v>
+      </c>
+      <c r="C22" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6216,456 +6305,456 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="40" t="n">
+      <c r="A5" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="41" t="n">
+      <c r="B5" s="42" t="n">
         <v>46283</v>
       </c>
       <c r="C5" s="19" t="n">
-        <v>1688</v>
+        <v>1120</v>
       </c>
       <c r="D5" s="22" t="n">
         <f aca="false">C5</f>
-        <v>1688</v>
+        <v>1120</v>
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="40" t="n">
+      <c r="A6" s="41" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="41" t="n">
+      <c r="B6" s="42" t="n">
         <v>46290</v>
       </c>
       <c r="C6" s="19" t="n">
-        <v>1320</v>
+        <v>880</v>
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">D5+C6</f>
-        <v>3008</v>
+        <v>2000</v>
       </c>
       <c r="E6" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="40" t="n">
+      <c r="A7" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="41" t="n">
+      <c r="B7" s="42" t="n">
         <v>46297</v>
       </c>
       <c r="C7" s="19" t="n">
-        <v>4672</v>
+        <v>2912</v>
       </c>
       <c r="D7" s="22" t="n">
         <f aca="false">D6+C7</f>
-        <v>7680</v>
+        <v>4912</v>
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="40" t="n">
+      <c r="A8" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="41" t="n">
+      <c r="B8" s="42" t="n">
         <v>46304</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>3360</v>
+        <v>2024</v>
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">D7+C8</f>
-        <v>11040</v>
+        <v>6936</v>
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="40" t="n">
+      <c r="A9" s="41" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="41" t="n">
+      <c r="B9" s="42" t="n">
         <v>46311</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>4785</v>
+        <v>2861</v>
       </c>
       <c r="D9" s="22" t="n">
         <f aca="false">D8+C9</f>
-        <v>15825</v>
+        <v>9797</v>
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="40" t="n">
+      <c r="A10" s="41" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="41" t="n">
+      <c r="B10" s="42" t="n">
         <v>46318</v>
       </c>
       <c r="C10" s="19" t="n">
-        <v>4002</v>
+        <v>2385</v>
       </c>
       <c r="D10" s="22" t="n">
         <f aca="false">D9+C10</f>
-        <v>19827</v>
+        <v>12182</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="40" t="n">
+      <c r="A11" s="41" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="41" t="n">
+      <c r="B11" s="42" t="n">
         <v>46325</v>
       </c>
       <c r="C11" s="19" t="n">
-        <v>5485</v>
+        <v>3299</v>
       </c>
       <c r="D11" s="22" t="n">
         <f aca="false">D10+C11</f>
-        <v>25312</v>
+        <v>15481</v>
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="40" t="n">
+      <c r="A12" s="41" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="41" t="n">
+      <c r="B12" s="42" t="n">
         <v>46332</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>4106</v>
+        <v>2495</v>
       </c>
       <c r="D12" s="22" t="n">
         <f aca="false">D11+C12</f>
-        <v>29418</v>
+        <v>17976</v>
       </c>
       <c r="E12" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="40" t="n">
+      <c r="A13" s="41" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="41" t="n">
+      <c r="B13" s="42" t="n">
         <v>46339</v>
       </c>
       <c r="C13" s="19" t="n">
-        <v>3893</v>
+        <v>2373</v>
       </c>
       <c r="D13" s="22" t="n">
         <f aca="false">D12+C13</f>
-        <v>33311</v>
+        <v>20349</v>
       </c>
       <c r="E13" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F13" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="40" t="n">
+      <c r="A14" s="41" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="41" t="n">
+      <c r="B14" s="42" t="n">
         <v>46346</v>
       </c>
       <c r="C14" s="19" t="n">
-        <v>3753</v>
+        <v>2275</v>
       </c>
       <c r="D14" s="22" t="n">
         <f aca="false">D13+C14</f>
-        <v>37064</v>
+        <v>22624</v>
       </c>
       <c r="E14" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F14" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="40" t="n">
+      <c r="A15" s="41" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="41" t="n">
+      <c r="B15" s="42" t="n">
         <v>46353</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>2320</v>
+        <v>1408</v>
       </c>
       <c r="D15" s="22" t="n">
         <f aca="false">D14+C15</f>
-        <v>39384</v>
+        <v>24032</v>
       </c>
       <c r="E15" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F15" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="40" t="n">
+      <c r="A16" s="41" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="41" t="n">
+      <c r="B16" s="42" t="n">
         <v>46360</v>
       </c>
       <c r="C16" s="19" t="n">
-        <v>2672</v>
+        <v>1664</v>
       </c>
       <c r="D16" s="22" t="n">
         <f aca="false">D15+C16</f>
-        <v>42056</v>
+        <v>25696</v>
       </c>
       <c r="E16" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F16" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="40" t="n">
+      <c r="A17" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="41" t="n">
+      <c r="B17" s="42" t="n">
         <v>46367</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>1508</v>
+        <v>1012</v>
       </c>
       <c r="D17" s="22" t="n">
         <f aca="false">D16+C17</f>
-        <v>43564</v>
+        <v>26708</v>
       </c>
       <c r="E17" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="40" t="n">
+      <c r="A18" s="41" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="41" t="n">
+      <c r="B18" s="42" t="n">
         <v>46374</v>
       </c>
       <c r="C18" s="19" t="n">
-        <v>3720</v>
+        <v>2696</v>
       </c>
       <c r="D18" s="22" t="n">
         <f aca="false">D17+C18</f>
-        <v>47284</v>
+        <v>29404</v>
       </c>
       <c r="E18" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F18" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="40" t="n">
+      <c r="A19" s="41" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="41" t="n">
+      <c r="B19" s="42" t="n">
         <v>46381</v>
       </c>
       <c r="C19" s="19" t="n">
-        <v>1850</v>
+        <v>1218</v>
       </c>
       <c r="D19" s="22" t="n">
         <f aca="false">D18+C19</f>
-        <v>49134</v>
+        <v>30622</v>
       </c>
       <c r="E19" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F19" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="40" t="n">
+      <c r="A20" s="41" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="41" t="n">
+      <c r="B20" s="42" t="n">
         <v>46388</v>
       </c>
       <c r="C20" s="19" t="n">
-        <v>3616</v>
+        <v>2240</v>
       </c>
       <c r="D20" s="22" t="n">
         <f aca="false">D19+C20</f>
-        <v>52750</v>
+        <v>32862</v>
       </c>
       <c r="E20" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F20" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="40" t="n">
+      <c r="A21" s="41" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="41" t="n">
+      <c r="B21" s="42" t="n">
         <v>46395</v>
       </c>
       <c r="C21" s="19" t="n">
-        <v>5004</v>
+        <v>3476</v>
       </c>
       <c r="D21" s="22" t="n">
         <f aca="false">D20+C21</f>
-        <v>57754</v>
+        <v>36338</v>
       </c>
       <c r="E21" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F21" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="40" t="n">
+      <c r="A22" s="41" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="41" t="n">
+      <c r="B22" s="42" t="n">
         <v>46402</v>
       </c>
       <c r="C22" s="19" t="n">
-        <v>2000</v>
+        <v>1200</v>
       </c>
       <c r="D22" s="22" t="n">
         <f aca="false">D21+C22</f>
-        <v>59754</v>
+        <v>37538</v>
       </c>
       <c r="E22" s="5" t="n">
         <f aca="false">Presupuesto!$B$15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="F22" s="5" t="n">
         <f aca="false">Presupuesto!$B$18</f>
-        <v>65393</v>
+        <v>42066</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="24" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B23" s="25"/>
       <c r="C23" s="27" t="n">
         <f aca="false">SUM(C5:C22)</f>
-        <v>59754</v>
+        <v>37538</v>
       </c>
       <c r="D23" s="24" t="str">
         <f aca="false">IF(ROUND(C23-Paquetes!V42,0)=0,"Cuadra con paquetes","Revisar")</f>
@@ -6676,7 +6765,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -6706,233 +6795,233 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="B5" s="42" t="n">
+        <v>240</v>
+      </c>
+      <c r="B5" s="43" t="n">
         <v>46332</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">Presupuesto!B15</f>
-        <v>62279</v>
+        <v>40063</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">INDEX('Curva S'!D5:D22,MATCH(B5,'Curva S'!B5:B22,0))</f>
-        <v>29418</v>
+        <v>17976</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="B8" s="38" t="n">
         <v>0.94</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">ROUND(B7*B8,0)</f>
-        <v>27653</v>
+        <v>16897</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="B10" s="35" t="n">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">ROUND(B9*B10,0)</f>
-        <v>29036</v>
+        <v>17911</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B12" s="22" t="n">
         <f aca="false">B9-B11</f>
-        <v>-1383</v>
+        <v>-1014</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="B13" s="22" t="n">
         <f aca="false">B9-B7</f>
-        <v>-1765</v>
+        <v>-1079</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="B14" s="43" t="n">
+        <v>258</v>
+      </c>
+      <c r="B14" s="44" t="n">
         <f aca="false">B9/B11</f>
-        <v>0.952369472379116</v>
+        <v>0.943386745575345</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="B15" s="43" t="n">
+        <v>260</v>
+      </c>
+      <c r="B15" s="44" t="n">
         <f aca="false">B9/B7</f>
-        <v>0.940002719423482</v>
+        <v>0.939975522919448</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">B6/B14</f>
-        <v>65393.7382562471</v>
+        <v>42467.206782269</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">B11+(B6-B9)</f>
-        <v>63662</v>
+        <v>41077</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="B18" s="22" t="n">
         <f aca="false">B11+(B6-B9)/(B14*B15)</f>
-        <v>67714.3330568935</v>
+        <v>44035.3044989092</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="B19" s="22" t="n">
         <f aca="false">B16-B11</f>
-        <v>36357.7382562471</v>
+        <v>24556.206782269</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">B6-B16</f>
-        <v>-3114.73825624706</v>
+        <v>-2404.20678226904</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="B21" s="43" t="n">
+        <v>272</v>
+      </c>
+      <c r="B21" s="44" t="n">
         <f aca="false">(B6-B9)/(B6-B11)</f>
-        <v>1.04160274343471</v>
+        <v>1.04577464788732</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="B23" s="13" t="str">
         <f aca="false">IF(B14&lt;1,"Sobrecosto: ","Dentro del costo: ")&amp;"CPI "&amp;TEXT(B14,"0.00")&amp;" · "&amp;IF(B15&lt;1,"Atraso: ","A tiempo: ")&amp;"SPI "&amp;TEXT(B15,"0.00")</f>
-        <v>Sobrecosto: CPI 0.95 · Atraso: SPI 0.94</v>
+        <v>Sobrecosto: CPI 0.94 · Atraso: SPI 0.94</v>
       </c>
     </row>
   </sheetData>
@@ -6961,12 +7050,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6974,185 +7063,185 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="B5" s="44" t="n">
+        <v>278</v>
+      </c>
+      <c r="B5" s="45" t="n">
         <v>216</v>
       </c>
-      <c r="C5" s="45" t="s">
-        <v>272</v>
+      <c r="C5" s="46" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B6" s="38" t="n">
         <v>0.15</v>
       </c>
-      <c r="C6" s="45" t="s">
-        <v>274</v>
+      <c r="C6" s="46" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="B7" s="46" t="n">
+        <v>282</v>
+      </c>
+      <c r="B7" s="47" t="n">
         <f aca="false">ROUND(B5*B6,0)</f>
         <v>32</v>
       </c>
-      <c r="C7" s="45" t="s">
-        <v>276</v>
+      <c r="C7" s="46" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="B8" s="47" t="n">
+        <v>284</v>
+      </c>
+      <c r="B8" s="40" t="n">
         <v>750</v>
       </c>
-      <c r="C8" s="45" t="s">
-        <v>278</v>
+      <c r="C8" s="46" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">B7*B8</f>
         <v>24000</v>
       </c>
-      <c r="C9" s="45" t="s">
-        <v>280</v>
+      <c r="C9" s="46" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="B10" s="47" t="n">
+        <v>288</v>
+      </c>
+      <c r="B10" s="40" t="n">
         <v>3600</v>
       </c>
-      <c r="C10" s="45" t="s">
-        <v>282</v>
+      <c r="C10" s="46" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">B9-B10</f>
         <v>20400</v>
       </c>
-      <c r="C11" s="45" t="s">
-        <v>284</v>
+      <c r="C11" s="46" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="B12" s="38" t="n">
         <v>0.1</v>
       </c>
-      <c r="C12" s="45" t="s">
-        <v>286</v>
+      <c r="C12" s="46" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="B13" s="5" t="n">
         <f aca="false">Presupuesto!B18</f>
-        <v>65393</v>
-      </c>
-      <c r="C13" s="45" t="s">
-        <v>211</v>
+        <v>42066</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">-B13+NPV(B12,B11,B11,B11)</f>
-        <v>-14661.2193839219</v>
-      </c>
-      <c r="C14" s="45" t="s">
-        <v>289</v>
+        <v>8665.78061607813</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="B15" s="22" t="n">
         <f aca="false">-B13+NPV(B12,B11,B11,B11,B11,B11)</f>
-        <v>11939.0500959323</v>
-      </c>
-      <c r="C15" s="45" t="s">
-        <v>291</v>
+        <v>35266.0500959323</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="B16" s="23" t="n">
         <f aca="false">(B11*5-B13)/B13</f>
-        <v>0.559799978590981</v>
-      </c>
-      <c r="C16" s="45" t="s">
-        <v>293</v>
+        <v>1.42476108971616</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="B17" s="48" t="n">
         <f aca="false">B13/B11</f>
-        <v>3.20553921568627</v>
-      </c>
-      <c r="C17" s="45" t="s">
-        <v>295</v>
+        <v>2.06205882352941</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="B18" s="5" t="n">
         <f aca="false">'No laborales'!C13+Presupuesto!B14+Presupuesto!B17</f>
-        <v>7849</v>
-      </c>
-      <c r="C18" s="45" t="s">
-        <v>297</v>
+        <v>6738</v>
+      </c>
+      <c r="C18" s="46" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B19" s="48" t="n">
         <f aca="false">B18/(B11/12)</f>
-        <v>4.61705882352941</v>
-      </c>
-      <c r="C19" s="45" t="s">
-        <v>299</v>
+        <v>3.96352941176471</v>
+      </c>
+      <c r="C19" s="46" t="s">
+        <v>306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restaura el acta v2 firmada y solo actualiza su presupuesto
El acta conserva su contenido y firmas; la sección 10 pasa a S/ 42 200
por entregable de la EDT, alineada con la línea base de costos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LWjTm2rp677phoNoYSvNSp
</commit_message>
<xml_diff>
--- a/docs/Costos_CRM_Essenza.xlsx
+++ b/docs/Costos_CRM_Essenza.xlsx
@@ -75,7 +75,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Monto de orden de magnitud aprobado en el acta ESSENZA-CRM-2026-001 (sección 10).</t>
+          <t xml:space="preserve">Monto de orden de magnitud aprobado en el acta ESSENZA-FID-2026-001 (sección 10).</t>
         </r>
       </text>
     </comment>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="306">
   <si>
     <t xml:space="preserve">Línea base de costos — CRM Predictivo y Retención Postventa · Essenza SPA</t>
   </si>
@@ -149,7 +149,7 @@
     <t xml:space="preserve">Línea base + reserva de gestión</t>
   </si>
   <si>
-    <t xml:space="preserve">Presupuesto autorizado en el acta (v3)</t>
+    <t xml:space="preserve">Presupuesto autorizado en el acta de constitución</t>
   </si>
   <si>
     <t xml:space="preserve">Orden de magnitud aprobado en el acta de constitución</t>
@@ -753,9 +753,6 @@
   </si>
   <si>
     <t xml:space="preserve">+ Reserva de gestión (S/)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presupuesto autorizado en el acta de constitución (v3)</t>
   </si>
   <si>
     <t xml:space="preserve">Holgura frente al acta (S/)</t>
@@ -1664,11 +1661,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="52922887"/>
-        <c:axId val="62129246"/>
+        <c:axId val="50411511"/>
+        <c:axId val="6687986"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="52922887"/>
+        <c:axId val="50411511"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1700,7 +1697,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62129246"/>
+        <c:crossAx val="6687986"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1708,7 +1705,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62129246"/>
+        <c:axId val="6687986"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1750,7 +1747,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52922887"/>
+        <c:crossAx val="50411511"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2370,11 +2367,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="60823393"/>
-        <c:axId val="77710426"/>
+        <c:axId val="51288020"/>
+        <c:axId val="65823511"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="60823393"/>
+        <c:axId val="51288020"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2406,7 +2403,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77710426"/>
+        <c:crossAx val="65823511"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2414,7 +2411,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77710426"/>
+        <c:axId val="65823511"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2490,7 +2487,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60823393"/>
+        <c:crossAx val="51288020"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6245,7 +6242,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>223</v>
+        <v>21</v>
       </c>
       <c r="B20" s="40" t="n">
         <v>42200</v>
@@ -6254,7 +6251,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B21" s="22" t="n">
         <f aca="false">B20-B18</f>
@@ -6267,7 +6264,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B22" s="22" t="n">
         <f aca="false">B20*1.1</f>
@@ -6305,32 +6302,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>232</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6765,7 +6762,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -6795,229 +6792,229 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B5" s="43" t="n">
         <v>46332</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">Presupuesto!B15</f>
         <v>40063</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">INDEX('Curva S'!D5:D22,MATCH(B5,'Curva S'!B5:B22,0))</f>
         <v>17976</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B8" s="38" t="n">
         <v>0.94</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">ROUND(B7*B8,0)</f>
         <v>16897</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B10" s="35" t="n">
         <v>1.06</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">ROUND(B9*B10,0)</f>
         <v>17911</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B12" s="22" t="n">
         <f aca="false">B9-B11</f>
         <v>-1014</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B13" s="22" t="n">
         <f aca="false">B9-B7</f>
         <v>-1079</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B14" s="44" t="n">
         <f aca="false">B9/B11</f>
         <v>0.943386745575345</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B15" s="44" t="n">
         <f aca="false">B9/B7</f>
         <v>0.939975522919448</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">B6/B14</f>
         <v>42467.206782269</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">B11+(B6-B9)</f>
         <v>41077</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B18" s="22" t="n">
         <f aca="false">B11+(B6-B9)/(B14*B15)</f>
         <v>44035.3044989092</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B19" s="22" t="n">
         <f aca="false">B16-B11</f>
         <v>24556.206782269</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">B6-B16</f>
         <v>-2404.20678226904</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B21" s="44" t="n">
         <f aca="false">(B6-B9)/(B6-B11)</f>
         <v>1.04577464788732</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B23" s="13" t="str">
         <f aca="false">IF(B14&lt;1,"Sobrecosto: ","Dentro del costo: ")&amp;"CPI "&amp;TEXT(B14,"0.00")&amp;" · "&amp;IF(B15&lt;1,"Atraso: ","A tiempo: ")&amp;"SPI "&amp;TEXT(B15,"0.00")</f>
@@ -7050,12 +7047,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7063,106 +7060,106 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B5" s="45" t="n">
         <v>216</v>
       </c>
       <c r="C5" s="46" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B6" s="38" t="n">
         <v>0.15</v>
       </c>
       <c r="C6" s="46" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B7" s="47" t="n">
         <f aca="false">ROUND(B5*B6,0)</f>
         <v>32</v>
       </c>
       <c r="C7" s="46" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B8" s="40" t="n">
         <v>750</v>
       </c>
       <c r="C8" s="46" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">B7*B8</f>
         <v>24000</v>
       </c>
       <c r="C9" s="46" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B10" s="40" t="n">
         <v>3600</v>
       </c>
       <c r="C10" s="46" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">B9-B10</f>
         <v>20400</v>
       </c>
       <c r="C11" s="46" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B12" s="38" t="n">
         <v>0.1</v>
       </c>
       <c r="C12" s="46" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B13" s="5" t="n">
         <f aca="false">Presupuesto!B18</f>
@@ -7174,74 +7171,74 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">-B13+NPV(B12,B11,B11,B11)</f>
         <v>8665.78061607813</v>
       </c>
       <c r="C14" s="46" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B15" s="22" t="n">
         <f aca="false">-B13+NPV(B12,B11,B11,B11,B11,B11)</f>
         <v>35266.0500959323</v>
       </c>
       <c r="C15" s="46" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B16" s="23" t="n">
         <f aca="false">(B11*5-B13)/B13</f>
         <v>1.42476108971616</v>
       </c>
       <c r="C16" s="46" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B17" s="48" t="n">
         <f aca="false">B13/B11</f>
         <v>2.06205882352941</v>
       </c>
       <c r="C17" s="46" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B18" s="5" t="n">
         <f aca="false">'No laborales'!C13+Presupuesto!B14+Presupuesto!B17</f>
         <v>6738</v>
       </c>
       <c r="C18" s="46" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B19" s="48" t="n">
         <f aca="false">B18/(B11/12)</f>
         <v>3.96352941176471</v>
       </c>
       <c r="C19" s="46" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revisión de concordancia entre secciones
- Fases del diccionario de la EDT alineadas con las fechas del cronograma.
- Responsables existentes en el equipo (sin 'líder técnico').
- Cronograma XML con tarifas por rol: MS Project muestra la misma mano de obra (S/ 35 096).
- Viabilidad: supuestos explícitos y vínculo con el caso de negocio del acta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LWjTm2rp677phoNoYSvNSp
</commit_message>
<xml_diff>
--- a/docs/Costos_CRM_Essenza.xlsx
+++ b/docs/Costos_CRM_Essenza.xlsx
@@ -920,7 +920,7 @@
     <t xml:space="preserve">Clientes en riesgo de abandono por año</t>
   </si>
   <si>
-    <t xml:space="preserve">Dato del análisis de la cartera (contexto del proyecto)</t>
+    <t xml:space="preserve">Supuesto del caso de negocio (≈ mitad de los 420 clientes); se valida con el modelo en H2</t>
   </si>
   <si>
     <t xml:space="preserve">Tasa de recuperación esperada</t>
@@ -938,7 +938,7 @@
     <t xml:space="preserve">Ingreso anual por cliente (S/)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ticket promedio anual por cliente (supuesto)</t>
+    <t xml:space="preserve">Gasto anual promedio por cliente (supuesto del caso de negocio)</t>
   </si>
   <si>
     <t xml:space="preserve">Beneficio bruto anual (S/)</t>
@@ -1661,11 +1661,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="50411511"/>
-        <c:axId val="6687986"/>
+        <c:axId val="13139669"/>
+        <c:axId val="5009372"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50411511"/>
+        <c:axId val="13139669"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1697,7 +1697,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6687986"/>
+        <c:crossAx val="5009372"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1705,7 +1705,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6687986"/>
+        <c:axId val="5009372"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1747,7 +1747,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50411511"/>
+        <c:crossAx val="13139669"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2367,11 +2367,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="51288020"/>
-        <c:axId val="65823511"/>
+        <c:axId val="86559902"/>
+        <c:axId val="37422479"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="51288020"/>
+        <c:axId val="86559902"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2403,7 +2403,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65823511"/>
+        <c:crossAx val="37422479"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2411,7 +2411,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="65823511"/>
+        <c:axId val="37422479"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2487,7 +2487,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51288020"/>
+        <c:crossAx val="86559902"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7066,7 +7066,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>277</v>
       </c>

</xml_diff>

<commit_message>
Alinea el texto del acta con el proyecto CRM conservando las firmas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LWjTm2rp677phoNoYSvNSp
</commit_message>
<xml_diff>
--- a/docs/Costos_CRM_Essenza.xlsx
+++ b/docs/Costos_CRM_Essenza.xlsx
@@ -75,7 +75,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Monto de orden de magnitud aprobado en el acta ESSENZA-FID-2026-001 (sección 10).</t>
+          <t xml:space="preserve">Monto de orden de magnitud aprobado en el acta ESSENZA-CRM-2026-001 (sección 10).</t>
         </r>
       </text>
     </comment>
@@ -1661,11 +1661,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="13139669"/>
-        <c:axId val="5009372"/>
+        <c:axId val="87143771"/>
+        <c:axId val="96519939"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="13139669"/>
+        <c:axId val="87143771"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1697,7 +1697,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5009372"/>
+        <c:crossAx val="96519939"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1705,7 +1705,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5009372"/>
+        <c:axId val="96519939"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1747,7 +1747,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13139669"/>
+        <c:crossAx val="87143771"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2367,11 +2367,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="86559902"/>
-        <c:axId val="37422479"/>
+        <c:axId val="26027227"/>
+        <c:axId val="58806481"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="86559902"/>
+        <c:axId val="26027227"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2403,7 +2403,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37422479"/>
+        <c:crossAx val="58806481"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2411,7 +2411,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="37422479"/>
+        <c:axId val="58806481"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2487,7 +2487,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86559902"/>
+        <c:crossAx val="26027227"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>